<commit_message>
#6 Fresh Client BOM and Deliverables generated after #7.
</commit_message>
<xml_diff>
--- a/Design Files/Powermodule-V7.0/BOM/Client BOM Powermodule-V7.0.xlsx
+++ b/Design Files/Powermodule-V7.0/BOM/Client BOM Powermodule-V7.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\gerholdvoorde-dronebms\Design Files\Powermodule-V7.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="196">
   <si>
     <t>#</t>
   </si>
@@ -87,12 +87,6 @@
     <t>C37, C38</t>
   </si>
   <si>
-    <t>D1, D4, D5, D6, D7</t>
-  </si>
-  <si>
-    <t>D2, D3</t>
-  </si>
-  <si>
     <t>J1</t>
   </si>
   <si>
@@ -144,9 +138,6 @@
     <t>R18, R20</t>
   </si>
   <si>
-    <t>R19, R22</t>
-  </si>
-  <si>
     <t>R24</t>
   </si>
   <si>
@@ -213,9 +204,6 @@
     <t>75V 200mW Single 1.25V@150mA 4ns 150mA SOD-323 Switching Diode ROHS</t>
   </si>
   <si>
-    <t>DIODE GEN PURP 100V 200MA SOD123</t>
-  </si>
-  <si>
     <t>CONN FFC BOTTOM 30POS 0.5MM R/A</t>
   </si>
   <si>
@@ -315,9 +303,6 @@
     <t>SOD-323</t>
   </si>
   <si>
-    <t>SOD-123</t>
-  </si>
-  <si>
     <t>FH12-30S-0.5SH(55)</t>
   </si>
   <si>
@@ -399,9 +384,6 @@
     <t>1N4148WS</t>
   </si>
   <si>
-    <t>MMSD4148T1G</t>
-  </si>
-  <si>
     <t>NCD0603G2</t>
   </si>
   <si>
@@ -474,9 +456,6 @@
     <t>Guangdong Hottech</t>
   </si>
   <si>
-    <t>ON Semiconductor</t>
-  </si>
-  <si>
     <t>Hirose</t>
   </si>
   <si>
@@ -619,6 +598,15 @@
   </si>
   <si>
     <t>Würth Elektronik</t>
+  </si>
+  <si>
+    <t>R19, R22, R29</t>
+  </si>
+  <si>
+    <t>D1, D4, D5</t>
+  </si>
+  <si>
+    <t>D2, D3, D6, D7</t>
   </si>
 </sst>
 </file>
@@ -959,9 +947,6 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -982,6 +967,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1270,7 +1258,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K45"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="7" customWidth="1"/>
@@ -1283,6 +1271,8 @@
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="29.42578125" customWidth="1"/>
+    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1294,9 +1284,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1310,25 +1300,25 @@
         <v>14</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="K2" s="8" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1337,26 +1327,26 @@
         <f>ROW(B3) - ROW($B$2)</f>
         <v>1</v>
       </c>
-      <c r="C3" s="28" t="s">
+      <c r="C3" s="27" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>15</v>
       </c>
       <c r="E3" s="16" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="J3" s="15">
         <v>15</v>
@@ -1369,26 +1359,26 @@
         <f t="shared" ref="B4:B43" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="27" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="17" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G4" s="18" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="I4" s="18" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="J4" s="17">
         <v>1</v>
@@ -1401,26 +1391,26 @@
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="27" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="I5" s="16" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="J5" s="15">
         <v>4</v>
@@ -1433,26 +1423,26 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="27" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>18</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G6" s="18" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I6" s="18" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="J6" s="17">
         <v>6</v>
@@ -1465,26 +1455,26 @@
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
-      <c r="C7" s="29" t="s">
+      <c r="C7" s="28" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="H7" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I7" s="16" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="J7" s="15">
         <v>5</v>
@@ -1497,26 +1487,26 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="28" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="17" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="J8" s="17">
         <v>4</v>
@@ -1529,26 +1519,26 @@
         <f>ROW(B9) - ROW($B$2)</f>
         <v>7</v>
       </c>
-      <c r="C9" s="29" t="s">
+      <c r="C9" s="28" t="s">
         <v>2</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>21</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="J9" s="15">
         <v>2</v>
@@ -1558,66 +1548,68 @@
     <row r="10" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="23">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B10" si="1">ROW(B10) - ROW($B$2)</f>
         <v>8</v>
       </c>
-      <c r="C10" s="28" t="s">
+      <c r="C10" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D10" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>125</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="I10" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="J10" s="17">
-        <v>5</v>
-      </c>
-      <c r="K10" s="17"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D10" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="H10" s="24" t="s">
+        <v>144</v>
+      </c>
+      <c r="I10" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="J10" s="24">
+        <v>3</v>
+      </c>
+      <c r="K10" s="26" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="23">
-        <f>ROW(B11) - ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C11" s="29" t="s">
+      <c r="C11" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="D11" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="F11" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="G11" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>151</v>
+      <c r="D11" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>144</v>
       </c>
       <c r="I11" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="J11" s="15">
-        <v>2</v>
-      </c>
-      <c r="K11" s="15"/>
+        <v>188</v>
+      </c>
+      <c r="J11" s="17">
+        <v>4</v>
+      </c>
+      <c r="K11" s="17"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
@@ -1625,26 +1617,26 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C12" s="28" t="s">
+      <c r="C12" s="27" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G12" s="18" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="I12" s="18" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J12" s="17">
         <v>1</v>
@@ -1657,26 +1649,26 @@
         <f>ROW(B13) - ROW($B$2)</f>
         <v>11</v>
       </c>
-      <c r="C13" s="29" t="s">
+      <c r="C13" s="28" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="I13" s="18" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J13" s="15">
         <v>1</v>
@@ -1689,26 +1681,26 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="28" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G14" s="18" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="I14" s="18" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J14" s="17">
         <v>1</v>
@@ -1721,26 +1713,26 @@
         <f>ROW(B15) - ROW($B$2)</f>
         <v>13</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>192</v>
+      <c r="C15" s="28" t="s">
+        <v>185</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="I15" s="16" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="J15" s="15">
         <v>1</v>
@@ -1753,26 +1745,26 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>192</v>
+      <c r="C16" s="28" t="s">
+        <v>185</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G16" s="18" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="I16" s="18" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="J16" s="17">
         <v>1</v>
@@ -1785,26 +1777,26 @@
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="29" t="s">
+      <c r="C17" s="28" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="I17" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J17" s="15">
         <v>3</v>
@@ -1817,26 +1809,26 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="28" t="s">
+      <c r="C18" s="27" t="s">
         <v>6</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G18" s="18" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="I18" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J18" s="17">
         <v>1</v>
@@ -1849,28 +1841,28 @@
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="29" t="s">
+      <c r="C19" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="31" t="s">
-        <v>72</v>
-      </c>
-      <c r="F19" s="30" t="s">
-        <v>194</v>
-      </c>
-      <c r="G19" s="31" t="s">
+      <c r="D19" s="29" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="F19" s="29" t="s">
+        <v>187</v>
+      </c>
+      <c r="G19" s="30" t="s">
         <v>7</v>
       </c>
-      <c r="H19" s="30" t="s">
-        <v>195</v>
+      <c r="H19" s="29" t="s">
+        <v>188</v>
       </c>
       <c r="I19" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="J19" s="30">
+        <v>188</v>
+      </c>
+      <c r="J19" s="29">
         <v>35</v>
       </c>
       <c r="K19" s="15"/>
@@ -1881,26 +1873,26 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="28" t="s">
+      <c r="C20" s="27" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G20" s="18" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H20" s="17" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="I20" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J20" s="17">
         <v>2</v>
@@ -1913,26 +1905,26 @@
         <f>ROW(B21) - ROW($B$2)</f>
         <v>19</v>
       </c>
-      <c r="C21" s="29" t="s">
-        <v>193</v>
+      <c r="C21" s="28" t="s">
+        <v>186</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="I21" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J21" s="15">
         <v>2</v>
@@ -1945,26 +1937,26 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C22" s="29" t="s">
+      <c r="C22" s="28" t="s">
         <v>9</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G22" s="18" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I22" s="18" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J22" s="17">
         <v>5</v>
@@ -1977,26 +1969,26 @@
         <f>ROW(B23) - ROW($B$2)</f>
         <v>21</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="C23" s="28" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I23" s="16" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="J23" s="15">
         <v>7</v>
@@ -2009,26 +2001,26 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C24" s="29" t="s">
+      <c r="C24" s="28" t="s">
         <v>9</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G24" s="18" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I24" s="18" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="J24" s="17">
         <v>1</v>
@@ -2041,26 +2033,26 @@
         <f>ROW(B25) - ROW($B$2)</f>
         <v>23</v>
       </c>
-      <c r="C25" s="29" t="s">
+      <c r="C25" s="28" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I25" s="16" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="J25" s="15">
         <v>3</v>
@@ -2073,31 +2065,33 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="D26" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="E26" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="F26" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="G26" s="18" t="s">
-        <v>135</v>
-      </c>
-      <c r="H26" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="I26" s="18" t="s">
-        <v>179</v>
-      </c>
-      <c r="J26" s="17">
+      <c r="D26" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="G26" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="I26" s="24" t="s">
+        <v>172</v>
+      </c>
+      <c r="J26" s="24">
         <v>1</v>
       </c>
-      <c r="K26" s="17"/>
+      <c r="K26" s="26" t="s">
+        <v>184</v>
+      </c>
     </row>
     <row r="27" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
@@ -2105,26 +2099,26 @@
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="C27" s="28" t="s">
         <v>9</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E27" s="16" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="H27" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I27" s="16" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="J27" s="15">
         <v>2</v>
@@ -2137,26 +2131,26 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" s="27" t="s">
         <v>9</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G28" s="18" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="H28" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I28" s="18" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="J28" s="17">
         <v>2</v>
@@ -2169,29 +2163,29 @@
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="15" t="s">
-        <v>41</v>
+      <c r="D29" s="17" t="s">
+        <v>193</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I29" s="16" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="J29" s="15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K29" s="15"/>
     </row>
@@ -2201,32 +2195,32 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C30" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="D30" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="E30" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="F30" s="25" t="s">
-        <v>106</v>
-      </c>
-      <c r="G30" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="H30" s="25" t="s">
-        <v>149</v>
-      </c>
-      <c r="I30" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="J30" s="25">
+      <c r="D30" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="F30" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="G30" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="H30" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="I30" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="J30" s="24">
         <v>1</v>
       </c>
-      <c r="K30" s="27" t="s">
-        <v>191</v>
+      <c r="K30" s="26" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2235,26 +2229,26 @@
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
-      <c r="C31" s="28" t="s">
+      <c r="C31" s="27" t="s">
         <v>9</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E31" s="16" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="I31" s="16" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="J31" s="15">
         <v>1</v>
@@ -2267,26 +2261,26 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C32" s="28" t="s">
+      <c r="C32" s="27" t="s">
         <v>9</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="H32" s="17" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="I32" s="18" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="J32" s="17">
         <v>3</v>
@@ -2299,26 +2293,26 @@
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
-      <c r="C33" s="29" t="s">
+      <c r="C33" s="28" t="s">
         <v>10</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E33" s="16" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J33" s="15">
         <v>1</v>
@@ -2331,32 +2325,32 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C34" s="28" t="s">
+      <c r="C34" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="25" t="s">
-        <v>46</v>
-      </c>
-      <c r="E34" s="26" t="s">
-        <v>85</v>
-      </c>
-      <c r="F34" s="25" t="s">
-        <v>194</v>
-      </c>
-      <c r="G34" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="H34" s="25" t="s">
-        <v>160</v>
-      </c>
-      <c r="I34" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="J34" s="25">
+      <c r="D34" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="F34" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="G34" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="H34" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="I34" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="J34" s="24">
         <v>1</v>
       </c>
-      <c r="K34" s="27" t="s">
-        <v>191</v>
+      <c r="K34" s="26" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2365,26 +2359,26 @@
         <f>ROW(B35) - ROW($B$2)</f>
         <v>33</v>
       </c>
-      <c r="C35" s="29" t="s">
+      <c r="C35" s="28" t="s">
         <v>11</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E35" s="16" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="H35" s="15" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I35" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J35" s="15">
         <v>1</v>
@@ -2397,26 +2391,26 @@
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C36" s="28" t="s">
+      <c r="C36" s="27" t="s">
         <v>11</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="H36" s="17" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="I36" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J36" s="17">
         <v>1</v>
@@ -2429,26 +2423,26 @@
         <f>ROW(B37) - ROW($B$2)</f>
         <v>35</v>
       </c>
-      <c r="C37" s="28" t="s">
+      <c r="C37" s="27" t="s">
         <v>11</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E37" s="16" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="I37" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J37" s="15">
         <v>1</v>
@@ -2461,26 +2455,26 @@
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C38" s="28" t="s">
+      <c r="C38" s="27" t="s">
         <v>11</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E38" s="18" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F38" s="17" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="G38" s="18" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H38" s="17" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="I38" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J38" s="17">
         <v>1</v>
@@ -2493,26 +2487,26 @@
         <f>ROW(B39) - ROW($B$2)</f>
         <v>37</v>
       </c>
-      <c r="C39" s="29" t="s">
+      <c r="C39" s="28" t="s">
         <v>11</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E39" s="16" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F39" s="15" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="H39" s="15" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="I39" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J39" s="15">
         <v>1</v>
@@ -2525,26 +2519,26 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C40" s="28" t="s">
+      <c r="C40" s="27" t="s">
         <v>12</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E40" s="18" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F40" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G40" s="18" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="H40" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="I40" s="16" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J40" s="17">
         <v>1</v>
@@ -2557,26 +2551,26 @@
         <f>ROW(B41) - ROW($B$2)</f>
         <v>39</v>
       </c>
-      <c r="C41" s="29" t="s">
+      <c r="C41" s="28" t="s">
         <v>13</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E41" s="16" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F41" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="H41" s="15" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="I41" s="16" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="J41" s="15">
         <v>1</v>
@@ -2589,26 +2583,26 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="27" t="s">
         <v>13</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F42" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G42" s="18" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="H42" s="17" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="I42" s="18" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="J42" s="17">
         <v>1</v>
@@ -2621,26 +2615,26 @@
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C43" s="28" t="s">
-        <v>196</v>
+      <c r="C43" s="27" t="s">
+        <v>189</v>
       </c>
       <c r="D43" s="17" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="E43" s="18" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="F43" s="17" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="G43" s="18" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="H43" s="17" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="I43" s="18" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="J43" s="17">
         <v>4</v>
@@ -2673,6 +2667,9 @@
       <c r="J45" s="4"/>
       <c r="K45" s="20"/>
     </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>

</xml_diff>